<commit_message>
Mejoras banco de semillas (fichas, UICN, origen, CSV)
</commit_message>
<xml_diff>
--- a/docs/recursos/fotos_faltantes_arboretum.xlsx
+++ b/docs/recursos/fotos_faltantes_arboretum.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fotos faltantes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisar nombres" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aves faltantes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisar nombres" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +72,18 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00888888"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -121,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -154,6 +167,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -519,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -667,6 +685,35 @@
       <c r="A23" s="2" t="inlineStr">
         <is>
           <t>• La fila 2 de la hoja "Fotos faltantes" es un EJEMPLO del formato esperado: borrala antes de empezar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Aves sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Se agregó la hoja «Aves faltantes» con 28 aves registradas que aún no tienen foto en el sitio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Al cargar el archivo en el Excel maestro (hoja Aves, columna "foto"), escribí el nombre EXACTO del archivo,</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>respetando mayúsculas/minúsculas y la extensión (.jpg / .JPG). En el sitio publicado, mayúsculas y minúsculas importan.</t>
         </is>
       </c>
     </row>
@@ -681,7 +728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2946,6 +2993,952 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>especie (nombre común)</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>nombre_cientifico</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>Buscar en Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>archivo</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>autor</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>licencia</t>
+        </is>
+      </c>
+      <c r="I1" s="12" t="inlineStr">
+        <is>
+          <t>url_imagen</t>
+        </is>
+      </c>
+      <c r="J1" s="12" t="inlineStr">
+        <is>
+          <t>listo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>(ej.)</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>Hornero</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>Furnarius rufus</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr">
+        <is>
+          <t>Hornero.jpg</t>
+        </is>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>Foto: A. Gómez (Wikimedia Commons)</t>
+        </is>
+      </c>
+      <c r="H2" s="13" t="inlineStr">
+        <is>
+          <t>CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="I2" s="13" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:...</t>
+        </is>
+      </c>
+      <c r="J2" s="13" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AVE003</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Biguá</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Nannopterum brasilianum</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AVE004</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cabecita negra</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Spinus magellanicus</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AVE007</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Carpintero campestre</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Colaptes campestris</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AVE008</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Chiflón</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Syrigma sibilatrix</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AVE011</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Colibrí común</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Chlorostilbon lucidus</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AVE012</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Colibrí garganta blanca</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Leucochloris albicollis</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AVE013</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Corbatita</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sporophila caerulescens</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>AVE014</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Cotorra</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Myiopsitta monachus</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AVE015</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cuervillo cara pelada</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Phimosus infuscatus</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AVE016</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Cuervillo de cañada</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Plegadis chihi</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AVE018</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Gaviota cocinera</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Larus dominicanus</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AVE019</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Golondrina</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Progne chalybea</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AVE020</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Golondrina tijerita</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Hirundo rustica</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AVE022</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Halcón aplomado</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Falco femoralis</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AVE023</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Halconcito colorado</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Falco sparverius</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>AVE025</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Jilguero</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Sicalis flaveola</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>AVE027</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Lechuza de campanario</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Tyto alba</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AVE028</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Milano blanco</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Elanus leucurus</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>AVE029</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Músico</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Agelaioides badius</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>AVE030</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Paloma doméstica</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Columba livia</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>AVE032</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Pecho colorado</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Leistes superciliaris</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>AVE034</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Piojito</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Serpophaga subcristata</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>AVE036</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Ratona</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Troglodytes aedon</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>AVE038</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Tacuarita azul</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Polioptila dumicola</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>AVE039</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Taguató</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Rupornis magnirostris</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>AVE042</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Torcacita</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Columbina picui</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>AVE044</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Tordo pico corto</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Molothrus bonariensis</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>AVE046</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Zorzal</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Turdus amaurochalinus</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>Buscar imágenes ▸</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>Ver especie ▸</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId58"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>